<commit_message>
Create packed app for str-analyzer
</commit_message>
<xml_diff>
--- a/str-analyzer/data/output_report.xlsx
+++ b/str-analyzer/data/output_report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/76717f10357f1721/Desktop/repos/aoi-reports/STR_Analyzer/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/76717f10357f1721/Desktop/repos/aoi-reports/str-analyzer/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="3" documentId="11_DEFC1C579F96349C51ABB726766DC45F3DDE1518" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90CDD858-289F-44D4-9CC4-16B6BE4C3FEC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Filtered Results" sheetId="1" r:id="rId1"/>
@@ -942,26 +942,6 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -1072,6 +1052,19 @@
             </c:numRef>
           </c:val>
           <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-32CF-4981-9191-1E57ADB0A02F}"/>
             </c:ext>
@@ -1365,26 +1358,6 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1497,562 +1470,6 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
@@ -2087,6 +1504,10 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>